<commit_message>
Added error checks for inorrect results from llm-judge and fixed annotations
</commit_message>
<xml_diff>
--- a/data/validation/annotation_workbook.xlsx
+++ b/data/validation/annotation_workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33119cfcffe101ac/Documents/Thesis/Thesis folder/conversational-group-rec-eval/data/validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="305" documentId="11_15E95FC385823942AC97A11103D4C0A7A638DA54" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DF82496-BC24-4EA2-9B97-3A9B8E81ABED}"/>
+  <xr:revisionPtr revIDLastSave="318" documentId="11_15E95FC385823942AC97A11103D4C0A7A638DA54" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84CD057C-B095-47E4-AFB4-00E5B518C8F4}"/>
   <bookViews>
-    <workbookView xWindow="9996" yWindow="0" windowWidth="13116" windowHeight="13776" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guidelines" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="124">
   <si>
     <t>Module 2 -- Human Annotation Workbook</t>
   </si>
@@ -372,9 +372,6 @@
   </si>
   <si>
     <t>times_repeated_before_ack</t>
-  </si>
-  <si>
-    <t>shifts - 1 or 2</t>
   </si>
   <si>
     <t>No</t>
@@ -506,10 +503,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1050,9 +1043,7 @@
       <c r="F2" s="6">
         <v>3</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>116</v>
-      </c>
+      <c r="G2" s="7"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
@@ -1062,7 +1053,7 @@
         <v>45</v>
       </c>
       <c r="C3" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="6">
         <v>1</v>
@@ -1083,7 +1074,7 @@
         <v>46</v>
       </c>
       <c r="C4" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D4" s="6">
         <v>2</v>
@@ -1125,7 +1116,7 @@
         <v>45</v>
       </c>
       <c r="C6" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="6">
         <v>2</v>
@@ -1230,7 +1221,7 @@
         <v>45</v>
       </c>
       <c r="C11" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="6">
         <v>2</v>
@@ -1251,7 +1242,7 @@
         <v>44</v>
       </c>
       <c r="C12" s="6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D12" s="6">
         <v>2</v>
@@ -1293,7 +1284,7 @@
         <v>46</v>
       </c>
       <c r="C14" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="6">
         <v>2</v>
@@ -1314,7 +1305,7 @@
         <v>44</v>
       </c>
       <c r="C15" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="6">
         <v>2</v>
@@ -1402,10 +1393,10 @@
         <v>53</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="F2" s="7"/>
     </row>
@@ -1420,10 +1411,10 @@
         <v>55</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F3" s="7"/>
     </row>
@@ -1438,10 +1429,10 @@
         <v>57</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F4" s="7"/>
     </row>
@@ -1456,7 +1447,7 @@
         <v>59</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E5" s="6"/>
       <c r="F5" s="7"/>
@@ -1472,10 +1463,10 @@
         <v>61</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F6" s="7"/>
     </row>
@@ -1490,10 +1481,10 @@
         <v>61</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F7" s="7"/>
     </row>
@@ -1508,10 +1499,10 @@
         <v>61</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F8" s="7"/>
     </row>
@@ -1526,7 +1517,7 @@
         <v>64</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E9" s="6"/>
       <c r="F9" s="7"/>
@@ -1542,10 +1533,10 @@
         <v>66</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F10" s="7"/>
     </row>
@@ -1560,7 +1551,7 @@
         <v>68</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="7"/>
@@ -1576,10 +1567,10 @@
         <v>66</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F12" s="7"/>
     </row>
@@ -1594,10 +1585,10 @@
         <v>71</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F13" s="7"/>
     </row>
@@ -1612,10 +1603,10 @@
         <v>73</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F14" s="7"/>
     </row>
@@ -1630,10 +1621,10 @@
         <v>73</v>
       </c>
       <c r="D15" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F15" s="7"/>
     </row>
@@ -1648,10 +1639,10 @@
         <v>73</v>
       </c>
       <c r="D16" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F16" s="7"/>
     </row>
@@ -1666,10 +1657,10 @@
         <v>74</v>
       </c>
       <c r="D17" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F17" s="7"/>
     </row>
@@ -1684,10 +1675,10 @@
         <v>73</v>
       </c>
       <c r="D18" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E18" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F18" s="7"/>
     </row>
@@ -1702,10 +1693,10 @@
         <v>74</v>
       </c>
       <c r="D19" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F19" s="7"/>
     </row>
@@ -1720,10 +1711,10 @@
         <v>73</v>
       </c>
       <c r="D20" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E20" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F20" s="7"/>
     </row>
@@ -1738,7 +1729,7 @@
         <v>55</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="7"/>
@@ -1754,10 +1745,10 @@
         <v>80</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F22" s="7"/>
     </row>
@@ -1772,10 +1763,10 @@
         <v>82</v>
       </c>
       <c r="D23" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F23" s="7"/>
     </row>
@@ -1790,10 +1781,10 @@
         <v>68</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F24" s="7"/>
     </row>
@@ -1808,10 +1799,10 @@
         <v>71</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F25" s="7"/>
     </row>
@@ -1826,10 +1817,10 @@
         <v>71</v>
       </c>
       <c r="D26" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F26" s="7"/>
     </row>
@@ -1844,10 +1835,10 @@
         <v>71</v>
       </c>
       <c r="D27" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F27" s="7"/>
     </row>
@@ -1862,10 +1853,10 @@
         <v>57</v>
       </c>
       <c r="D28" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F28" s="7"/>
     </row>
@@ -1880,10 +1871,10 @@
         <v>57</v>
       </c>
       <c r="D29" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F29" s="7"/>
     </row>
@@ -1898,10 +1889,10 @@
         <v>64</v>
       </c>
       <c r="D30" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F30" s="7"/>
     </row>
@@ -1916,10 +1907,10 @@
         <v>84</v>
       </c>
       <c r="D31" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F31" s="7"/>
     </row>
@@ -1934,10 +1925,10 @@
         <v>84</v>
       </c>
       <c r="D32" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F32" s="7"/>
     </row>
@@ -1952,7 +1943,7 @@
         <v>71</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="7"/>
@@ -1968,10 +1959,10 @@
         <v>87</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F34" s="7"/>
     </row>
@@ -1986,10 +1977,10 @@
         <v>74</v>
       </c>
       <c r="D35" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F35" s="7"/>
     </row>
@@ -2004,10 +1995,10 @@
         <v>89</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F36" s="7"/>
     </row>
@@ -2022,10 +2013,10 @@
         <v>74</v>
       </c>
       <c r="D37" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F37" s="7"/>
     </row>
@@ -2040,10 +2031,10 @@
         <v>91</v>
       </c>
       <c r="D38" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E38" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F38" s="7"/>
     </row>
@@ -2058,10 +2049,10 @@
         <v>91</v>
       </c>
       <c r="D39" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F39" s="7"/>
     </row>
@@ -2076,10 +2067,10 @@
         <v>71</v>
       </c>
       <c r="D40" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F40" s="7"/>
     </row>
@@ -2094,10 +2085,10 @@
         <v>71</v>
       </c>
       <c r="D41" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E41" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F41" s="7"/>
     </row>
@@ -2112,10 +2103,10 @@
         <v>71</v>
       </c>
       <c r="D42" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F42" s="7"/>
     </row>
@@ -2130,10 +2121,10 @@
         <v>53</v>
       </c>
       <c r="D43" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E43" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F43" s="7"/>
     </row>
@@ -2148,10 +2139,10 @@
         <v>53</v>
       </c>
       <c r="D44" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F44" s="7"/>
     </row>
@@ -2166,10 +2157,10 @@
         <v>68</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F45" s="7"/>
     </row>
@@ -2184,10 +2175,10 @@
         <v>66</v>
       </c>
       <c r="D46" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E46" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F46" s="7"/>
     </row>
@@ -2202,10 +2193,10 @@
         <v>66</v>
       </c>
       <c r="D47" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F47" s="7"/>
     </row>
@@ -2220,10 +2211,10 @@
         <v>96</v>
       </c>
       <c r="D48" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F48" s="7"/>
     </row>
@@ -2238,10 +2229,10 @@
         <v>87</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F49" s="7"/>
     </row>
@@ -2256,10 +2247,10 @@
         <v>91</v>
       </c>
       <c r="D50" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F50" s="7"/>
     </row>
@@ -2274,10 +2265,10 @@
         <v>97</v>
       </c>
       <c r="D51" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F51" s="7"/>
     </row>
@@ -2292,10 +2283,10 @@
         <v>80</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F52" s="7"/>
     </row>
@@ -2310,10 +2301,10 @@
         <v>87</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F53" s="7"/>
     </row>
@@ -2328,10 +2319,10 @@
         <v>99</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F54" s="7"/>
     </row>
@@ -2346,10 +2337,10 @@
         <v>99</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F55" s="7"/>
     </row>
@@ -2364,10 +2355,10 @@
         <v>87</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F56" s="7"/>
     </row>
@@ -2382,10 +2373,10 @@
         <v>66</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F57" s="7"/>
     </row>
@@ -2400,7 +2391,7 @@
         <v>101</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E58" s="6"/>
       <c r="F58" s="7"/>
@@ -2416,7 +2407,7 @@
         <v>84</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E59" s="6"/>
       <c r="F59" s="7"/>
@@ -2432,10 +2423,10 @@
         <v>64</v>
       </c>
       <c r="D60" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E60" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F60" s="7"/>
     </row>
@@ -2450,7 +2441,7 @@
         <v>102</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E61" s="6"/>
       <c r="F61" s="7"/>
@@ -2466,7 +2457,7 @@
         <v>61</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E62" s="6"/>
       <c r="F62" s="7"/>
@@ -2482,7 +2473,7 @@
         <v>89</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E63" s="6"/>
       <c r="F63" s="7"/>
@@ -2498,10 +2489,10 @@
         <v>103</v>
       </c>
       <c r="D64" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F64" s="7"/>
     </row>
@@ -2516,10 +2507,10 @@
         <v>103</v>
       </c>
       <c r="D65" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E65" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F65" s="7"/>
     </row>
@@ -2534,10 +2525,10 @@
         <v>101</v>
       </c>
       <c r="D66" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E66" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F66" s="7"/>
     </row>
@@ -2552,7 +2543,7 @@
         <v>101</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E67" s="6"/>
       <c r="F67" s="7"/>
@@ -2568,7 +2559,7 @@
         <v>73</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E68" s="6"/>
       <c r="F68" s="7"/>
@@ -2584,10 +2575,10 @@
         <v>103</v>
       </c>
       <c r="D69" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F69" s="7"/>
     </row>
@@ -2602,10 +2593,10 @@
         <v>68</v>
       </c>
       <c r="D70" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E70" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E70" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F70" s="7"/>
     </row>
@@ -2620,10 +2611,10 @@
         <v>102</v>
       </c>
       <c r="D71" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E71" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F71" s="7"/>
     </row>
@@ -2638,10 +2629,10 @@
         <v>84</v>
       </c>
       <c r="D72" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E72" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E72" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F72" s="7"/>
     </row>
@@ -2656,10 +2647,10 @@
         <v>96</v>
       </c>
       <c r="D73" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E73" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E73" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F73" s="7"/>
     </row>
@@ -2674,10 +2665,10 @@
         <v>101</v>
       </c>
       <c r="D74" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E74" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F74" s="7"/>
     </row>
@@ -2692,10 +2683,10 @@
         <v>101</v>
       </c>
       <c r="D75" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E75" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E75" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F75" s="7"/>
     </row>
@@ -2710,10 +2701,10 @@
         <v>103</v>
       </c>
       <c r="D76" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E76" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F76" s="7"/>
     </row>
@@ -2728,10 +2719,10 @@
         <v>106</v>
       </c>
       <c r="D77" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E77" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F77" s="7"/>
     </row>
@@ -2746,7 +2737,7 @@
         <v>80</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E78" s="6"/>
       <c r="F78" s="7"/>
@@ -2762,7 +2753,7 @@
         <v>74</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E79" s="6"/>
       <c r="F79" s="7"/>
@@ -2778,10 +2769,10 @@
         <v>55</v>
       </c>
       <c r="D80" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E80" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E80" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F80" s="7"/>
     </row>
@@ -2796,10 +2787,10 @@
         <v>87</v>
       </c>
       <c r="D81" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E81" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E81" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F81" s="7"/>
     </row>
@@ -2814,10 +2805,10 @@
         <v>87</v>
       </c>
       <c r="D82" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E82" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F82" s="7"/>
     </row>
@@ -2832,10 +2823,10 @@
         <v>82</v>
       </c>
       <c r="D83" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E83" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E83" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F83" s="7"/>
     </row>
@@ -2850,7 +2841,7 @@
         <v>91</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E84" s="6"/>
       <c r="F84" s="7"/>
@@ -2866,10 +2857,10 @@
         <v>74</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F85" s="7"/>
     </row>
@@ -2884,10 +2875,10 @@
         <v>97</v>
       </c>
       <c r="D86" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E86" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E86" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F86" s="7"/>
     </row>
@@ -2902,10 +2893,10 @@
         <v>97</v>
       </c>
       <c r="D87" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E87" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E87" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F87" s="7"/>
     </row>
@@ -2920,10 +2911,10 @@
         <v>68</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F88" s="7"/>
     </row>
@@ -2938,10 +2929,10 @@
         <v>97</v>
       </c>
       <c r="D89" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E89" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E89" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F89" s="7"/>
     </row>
@@ -2956,10 +2947,10 @@
         <v>110</v>
       </c>
       <c r="D90" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E90" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E90" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F90" s="7"/>
     </row>
@@ -2974,10 +2965,10 @@
         <v>110</v>
       </c>
       <c r="D91" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E91" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E91" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F91" s="7"/>
     </row>
@@ -2992,10 +2983,10 @@
         <v>106</v>
       </c>
       <c r="D92" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E92" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E92" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F92" s="7"/>
     </row>
@@ -3010,10 +3001,10 @@
         <v>53</v>
       </c>
       <c r="D93" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E93" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E93" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F93" s="7"/>
     </row>
@@ -3028,10 +3019,10 @@
         <v>102</v>
       </c>
       <c r="D94" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E94" s="6" t="s">
         <v>119</v>
-      </c>
-      <c r="E94" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="F94" s="7"/>
     </row>
@@ -3046,15 +3037,15 @@
         <v>87</v>
       </c>
       <c r="D95" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E95" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E95" s="6" t="s">
-        <v>120</v>
-      </c>
       <c r="F95" s="7"/>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="2">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown list." sqref="D2:D95" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
@@ -3119,7 +3110,7 @@
         <v>2</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G2" s="7"/>
     </row>
@@ -3140,7 +3131,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G3" s="7"/>
     </row>
@@ -3161,7 +3152,7 @@
         <v>5</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G4" s="7"/>
     </row>
@@ -3182,7 +3173,7 @@
         <v>8</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G5" s="7"/>
     </row>
@@ -3203,7 +3194,7 @@
         <v>9</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G6" s="7"/>
     </row>
@@ -3224,7 +3215,7 @@
         <v>2</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G7" s="7"/>
     </row>
@@ -3245,7 +3236,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G8" s="7"/>
     </row>
@@ -3266,7 +3257,7 @@
         <v>4</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G9" s="7"/>
     </row>
@@ -3287,7 +3278,7 @@
         <v>9</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G10" s="7"/>
     </row>
@@ -3308,7 +3299,7 @@
         <v>3</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G11" s="7"/>
     </row>
@@ -3329,7 +3320,7 @@
         <v>4</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G12" s="7"/>
     </row>
@@ -3350,7 +3341,7 @@
         <v>5</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G13" s="7"/>
     </row>
@@ -3371,7 +3362,7 @@
         <v>8</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G14" s="7"/>
     </row>
@@ -3392,7 +3383,7 @@
         <v>9</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G15" s="7"/>
     </row>
@@ -3413,7 +3404,7 @@
         <v>11</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G16" s="7"/>
     </row>
@@ -3434,7 +3425,7 @@
         <v>6</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G17" s="7"/>
     </row>
@@ -3455,7 +3446,7 @@
         <v>7</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G18" s="7"/>
     </row>
@@ -3476,7 +3467,7 @@
         <v>11</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G19" s="7"/>
     </row>
@@ -3497,7 +3488,7 @@
         <v>2</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G20" s="7"/>
     </row>
@@ -3518,7 +3509,7 @@
         <v>2</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G21" s="7"/>
     </row>
@@ -3539,7 +3530,7 @@
         <v>8</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G22" s="7"/>
     </row>
@@ -3560,7 +3551,7 @@
         <v>8</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G23" s="7"/>
     </row>
@@ -3581,7 +3572,7 @@
         <v>2</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G24" s="7"/>
     </row>
@@ -3602,7 +3593,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G25" s="7"/>
     </row>
@@ -3623,7 +3614,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G26" s="7"/>
     </row>
@@ -3644,7 +3635,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G27" s="7"/>
     </row>
@@ -3665,7 +3656,7 @@
         <v>3</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G28" s="7"/>
     </row>
@@ -3686,7 +3677,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G29" s="7"/>
     </row>
@@ -3707,7 +3698,7 @@
         <v>2</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G30" s="7"/>
     </row>
@@ -3728,7 +3719,7 @@
         <v>3</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G31" s="7"/>
     </row>
@@ -3749,7 +3740,7 @@
         <v>2</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G32" s="7"/>
     </row>
@@ -3770,7 +3761,7 @@
         <v>2</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G33" s="7"/>
     </row>
@@ -3791,7 +3782,7 @@
         <v>2</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G34" s="7"/>
     </row>
@@ -3812,7 +3803,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G35" s="7"/>
     </row>
@@ -3833,7 +3824,7 @@
         <v>3</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G36" s="7"/>
     </row>
@@ -3854,7 +3845,7 @@
         <v>2</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G37" s="7"/>
     </row>
@@ -3875,7 +3866,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G38" s="7"/>
     </row>
@@ -3896,7 +3887,7 @@
         <v>2</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G39" s="7"/>
     </row>
@@ -3917,7 +3908,7 @@
         <v>2</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G40" s="7"/>
     </row>
@@ -3938,7 +3929,7 @@
         <v>2</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G41" s="7"/>
     </row>
@@ -3959,7 +3950,7 @@
         <v>3</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G42" s="7"/>
     </row>
@@ -3980,7 +3971,7 @@
         <v>3</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G43" s="7"/>
     </row>
@@ -4001,7 +3992,7 @@
         <v>2</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G44" s="7"/>
     </row>
@@ -4022,7 +4013,7 @@
         <v>3</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G45" s="7"/>
     </row>
@@ -4043,7 +4034,7 @@
         <v>2</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G46" s="7"/>
     </row>
@@ -4064,7 +4055,7 @@
         <v>2</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G47" s="7"/>
     </row>
@@ -4085,7 +4076,7 @@
         <v>3</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G48" s="7"/>
     </row>
@@ -4106,7 +4097,7 @@
         <v>2</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G49" s="7"/>
     </row>
@@ -4127,7 +4118,7 @@
         <v>3</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G50" s="7"/>
     </row>
@@ -4148,7 +4139,7 @@
         <v>4</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G51" s="7"/>
     </row>
@@ -4169,7 +4160,7 @@
         <v>6</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G52" s="7"/>
     </row>
@@ -4190,7 +4181,7 @@
         <v>7</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G53" s="7"/>
     </row>
@@ -4211,7 +4202,7 @@
         <v>8</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G54" s="7"/>
     </row>
@@ -4232,7 +4223,7 @@
         <v>9</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G55" s="7"/>
     </row>
@@ -4253,7 +4244,7 @@
         <v>10</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G56" s="7"/>
     </row>
@@ -4274,7 +4265,7 @@
         <v>11</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G57" s="7"/>
     </row>
@@ -4295,7 +4286,7 @@
         <v>12</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G58" s="7"/>
     </row>
@@ -4316,7 +4307,7 @@
         <v>13</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G59" s="7"/>
     </row>
@@ -4337,7 +4328,7 @@
         <v>14</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G60" s="7"/>
     </row>
@@ -4358,7 +4349,7 @@
         <v>15</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G61" s="7"/>
     </row>
@@ -4379,7 +4370,7 @@
         <v>2</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G62" s="7"/>
     </row>
@@ -4400,7 +4391,7 @@
         <v>7</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G63" s="7"/>
     </row>
@@ -4421,7 +4412,7 @@
         <v>8</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G64" s="7"/>
     </row>
@@ -4442,7 +4433,7 @@
         <v>2</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G65" s="7"/>
     </row>
@@ -4463,7 +4454,7 @@
         <v>7</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G66" s="7"/>
     </row>
@@ -4484,7 +4475,7 @@
         <v>8</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G67" s="7"/>
     </row>
@@ -4505,7 +4496,7 @@
         <v>10</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G68" s="7"/>
     </row>
@@ -4526,7 +4517,7 @@
         <v>14</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G69" s="7"/>
     </row>
@@ -4547,7 +4538,7 @@
         <v>15</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G70" s="7"/>
     </row>
@@ -4568,7 +4559,7 @@
         <v>16</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G71" s="7"/>
     </row>
@@ -4589,7 +4580,7 @@
         <v>3</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G72" s="7"/>
     </row>
@@ -4610,7 +4601,7 @@
         <v>5</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G73" s="7"/>
     </row>
@@ -4631,7 +4622,7 @@
         <v>10</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G74" s="7"/>
     </row>
@@ -4652,7 +4643,7 @@
         <v>2</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G75" s="7"/>
     </row>
@@ -4673,7 +4664,7 @@
         <v>4</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G76" s="7"/>
     </row>
@@ -4694,7 +4685,7 @@
         <v>5</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G77" s="7"/>
     </row>
@@ -4715,7 +4706,7 @@
         <v>6</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G78" s="7"/>
     </row>
@@ -4736,7 +4727,7 @@
         <v>7</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G79" s="7"/>
     </row>
@@ -4757,7 +4748,7 @@
         <v>8</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G80" s="7"/>
     </row>
@@ -4778,7 +4769,7 @@
         <v>13</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G81" s="7"/>
     </row>
@@ -4799,7 +4790,7 @@
         <v>14</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G82" s="7"/>
     </row>
@@ -4820,7 +4811,7 @@
         <v>2</v>
       </c>
       <c r="F83" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G83" s="7"/>
     </row>
@@ -4841,7 +4832,7 @@
         <v>3</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G84" s="7"/>
     </row>
@@ -4862,7 +4853,7 @@
         <v>6</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G85" s="7"/>
     </row>
@@ -4883,7 +4874,7 @@
         <v>8</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G86" s="7"/>
     </row>
@@ -4904,7 +4895,7 @@
         <v>9</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G87" s="7"/>
     </row>
@@ -4925,7 +4916,7 @@
         <v>10</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G88" s="7"/>
     </row>
@@ -4946,7 +4937,7 @@
         <v>13</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G89" s="7"/>
     </row>
@@ -4967,7 +4958,7 @@
         <v>14</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G90" s="7"/>
     </row>
@@ -4988,7 +4979,7 @@
         <v>2</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G91" s="7"/>
     </row>
@@ -5009,7 +5000,7 @@
         <v>2</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G92" s="7"/>
     </row>
@@ -5030,7 +5021,7 @@
         <v>2</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G93" s="7"/>
     </row>
@@ -5051,7 +5042,7 @@
         <v>2</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G94" s="7"/>
     </row>
@@ -5072,7 +5063,7 @@
         <v>2</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G95" s="7"/>
     </row>
@@ -5093,7 +5084,7 @@
         <v>2</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G96" s="7"/>
     </row>
@@ -5114,7 +5105,7 @@
         <v>2</v>
       </c>
       <c r="F97" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G97" s="7"/>
     </row>
@@ -5135,7 +5126,7 @@
         <v>2</v>
       </c>
       <c r="F98" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G98" s="7"/>
     </row>
@@ -5156,7 +5147,7 @@
         <v>3</v>
       </c>
       <c r="F99" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G99" s="7"/>
     </row>
@@ -5177,7 +5168,7 @@
         <v>2</v>
       </c>
       <c r="F100" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G100" s="7"/>
     </row>
@@ -5198,7 +5189,7 @@
         <v>3</v>
       </c>
       <c r="F101" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G101" s="7"/>
     </row>
@@ -5219,7 +5210,7 @@
         <v>4</v>
       </c>
       <c r="F102" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G102" s="7"/>
     </row>
@@ -5240,7 +5231,7 @@
         <v>5</v>
       </c>
       <c r="F103" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G103" s="7"/>
     </row>
@@ -5261,7 +5252,7 @@
         <v>2</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G104" s="7"/>
     </row>
@@ -5282,7 +5273,7 @@
         <v>2</v>
       </c>
       <c r="F105" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G105" s="7"/>
     </row>
@@ -5303,7 +5294,7 @@
         <v>2</v>
       </c>
       <c r="F106" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G106" s="7"/>
     </row>
@@ -5324,7 +5315,7 @@
         <v>4</v>
       </c>
       <c r="F107" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G107" s="7"/>
     </row>
@@ -5345,7 +5336,7 @@
         <v>2</v>
       </c>
       <c r="F108" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G108" s="7"/>
     </row>
@@ -5366,7 +5357,7 @@
         <v>4</v>
       </c>
       <c r="F109" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G109" s="7"/>
     </row>
@@ -5387,7 +5378,7 @@
         <v>2</v>
       </c>
       <c r="F110" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G110" s="7"/>
     </row>
@@ -5408,7 +5399,7 @@
         <v>2</v>
       </c>
       <c r="F111" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G111" s="7"/>
     </row>
@@ -5429,7 +5420,7 @@
         <v>2</v>
       </c>
       <c r="F112" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G112" s="7"/>
     </row>
@@ -5450,7 +5441,7 @@
         <v>2</v>
       </c>
       <c r="F113" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G113" s="7"/>
     </row>
@@ -5471,7 +5462,7 @@
         <v>2</v>
       </c>
       <c r="F114" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G114" s="7"/>
     </row>
@@ -5492,7 +5483,7 @@
         <v>2</v>
       </c>
       <c r="F115" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G115" s="7"/>
     </row>
@@ -5513,7 +5504,7 @@
         <v>2</v>
       </c>
       <c r="F116" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G116" s="7"/>
     </row>
@@ -5534,7 +5525,7 @@
         <v>2</v>
       </c>
       <c r="F117" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G117" s="7"/>
     </row>
@@ -5555,7 +5546,7 @@
         <v>2</v>
       </c>
       <c r="F118" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G118" s="7"/>
     </row>

</xml_diff>